<commit_message>
Sample data: use invented New Zealand-style place names
</commit_message>
<xml_diff>
--- a/sample/supervisor_schedule.xlsx
+++ b/sample/supervisor_schedule.xlsx
@@ -449,7 +449,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
     <row r="676">
       <c r="A676" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
     <row r="678">
       <c r="A678" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
     <row r="720">
       <c r="A720" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3216,7 @@
     <row r="722">
       <c r="A722" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
     <row r="724">
       <c r="A724" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
     <row r="743">
       <c r="A743" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3305,7 @@
     <row r="745">
       <c r="A745" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3313,7 @@
     <row r="747">
       <c r="A747" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey and Finley./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey and Finley./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
     <row r="768">
       <c r="A768" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
     <row r="770">
       <c r="A770" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
     <row r="789">
       <c r="A789" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
     <row r="791">
       <c r="A791" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
     <row r="793">
       <c r="A793" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
     <row r="812">
       <c r="A812" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
     <row r="814">
       <c r="A814" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
     <row r="837">
       <c r="A837" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
     <row r="908">
       <c r="A908" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
     <row r="927">
       <c r="A927" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4017,7 @@
     <row r="929">
       <c r="A929" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
     <row r="931">
       <c r="A931" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
     <row r="950">
       <c r="A950" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
     <row r="952">
       <c r="A952" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
     <row r="954">
       <c r="A954" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
     <row r="975">
       <c r="A975" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
     <row r="996">
       <c r="A996" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
     <row r="998">
       <c r="A998" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
     <row r="1000">
       <c r="A1000" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
     <row r="1019">
       <c r="A1019" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
     <row r="1021">
       <c r="A1021" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
     <row r="1023">
       <c r="A1023" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
     <row r="1042">
       <c r="A1042" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
     <row r="1046">
       <c r="A1046" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
     <row r="1065">
       <c r="A1065" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
     <row r="1069">
       <c r="A1069" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
     <row r="1088">
       <c r="A1088" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
     <row r="1090">
       <c r="A1090" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
     <row r="1092">
       <c r="A1092" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
     <row r="1111">
       <c r="A1111" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4729,7 @@
     <row r="1113">
       <c r="A1113" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4810,7 @@
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
     <row r="1136">
       <c r="A1136" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
     <row r="1138">
       <c r="A1138" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4899,7 @@
     <row r="1157">
       <c r="A1157" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
     <row r="1159">
       <c r="A1159" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4915,7 +4915,7 @@
     <row r="1161">
       <c r="A1161" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5085,7 +5085,7 @@
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5093,7 @@
     <row r="1207">
       <c r="A1207" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
     <row r="1230">
       <c r="A1230" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
     <row r="1249">
       <c r="A1249" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
     <row r="1251">
       <c r="A1251" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
     <row r="1253">
       <c r="A1253" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5344,7 @@
     <row r="1272">
       <c r="A1272" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
     <row r="1274">
       <c r="A1274" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
     <row r="1276">
       <c r="A1276" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Casey and Finley./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Casey and Finley./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5433,7 @@
     <row r="1295">
       <c r="A1295" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
     <row r="1297">
       <c r="A1297" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake and Emery./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake and Emery./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
     <row r="1299">
       <c r="A1299" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
     <row r="1318">
       <c r="A1318" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
     <row r="1320">
       <c r="A1320" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5538,7 @@
     <row r="1322">
       <c r="A1322" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
     <row r="1341">
       <c r="A1341" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5619,7 @@
     <row r="1343">
       <c r="A1343" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
     <row r="1364">
       <c r="A1364" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
     <row r="1366">
       <c r="A1366" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
     <row r="1368">
       <c r="A1368" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5789,7 +5789,7 @@
     <row r="1387">
       <c r="A1387" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5797,7 @@
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5805,7 +5805,7 @@
     <row r="1391">
       <c r="A1391" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5878,7 @@
     <row r="1410">
       <c r="A1410" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5886,7 +5886,7 @@
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5894,7 @@
     <row r="1414">
       <c r="A1414" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5967,7 @@
     <row r="1433">
       <c r="A1433" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake and Emery./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake and Emery./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5983,7 @@
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
     <row r="1456">
       <c r="A1456" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6064,7 @@
     <row r="1458">
       <c r="A1458" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
     <row r="1460">
       <c r="A1460" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
     <row r="1481">
       <c r="A1481" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sample data: invented New Zealand-style place names
Co-authored-by: Rimsha Shakya <rimshashakya11-dotcom@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/sample/supervisor_schedule.xlsx
+++ b/sample/supervisor_schedule.xlsx
@@ -449,7 +449,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -465,7 +465,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -538,7 +538,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -554,7 +554,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -635,7 +635,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -643,7 +643,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -732,7 +732,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -805,7 +805,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -813,7 +813,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -894,7 +894,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -910,7 +910,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -999,7 +999,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1072,7 +1072,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1080,7 +1080,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1088,7 +1088,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1169,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1177,7 +1177,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1250,7 +1250,7 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1266,7 +1266,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1339,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1347,7 +1347,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1428,7 +1428,7 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1444,7 +1444,7 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1517,7 +1517,7 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1533,7 +1533,7 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -1606,7 +1606,7 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1695,7 +1695,7 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1703,7 +1703,7 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1711,7 +1711,7 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1784,7 +1784,7 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1792,7 +1792,7 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1800,7 +1800,7 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1873,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -1881,7 +1881,7 @@
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -1889,7 +1889,7 @@
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -1970,7 +1970,7 @@
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -1978,7 +1978,7 @@
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2051,7 +2051,7 @@
     <row r="421">
       <c r="A421" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
     <row r="423">
       <c r="A423" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2067,7 @@
     <row r="425">
       <c r="A425" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
     <row r="444">
       <c r="A444" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2148,7 +2148,7 @@
     <row r="446">
       <c r="A446" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2156,7 +2156,7 @@
     <row r="448">
       <c r="A448" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2229,7 +2229,7 @@
     <row r="467">
       <c r="A467" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2237,7 +2237,7 @@
     <row r="469">
       <c r="A469" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2245,7 +2245,7 @@
     <row r="471">
       <c r="A471" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2318,7 +2318,7 @@
     <row r="490">
       <c r="A490" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2326,7 @@
     <row r="492">
       <c r="A492" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2334,7 @@
     <row r="494">
       <c r="A494" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2407,7 @@
     <row r="513">
       <c r="A513" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
     <row r="515">
       <c r="A515" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2423,7 +2423,7 @@
     <row r="517">
       <c r="A517" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2496,7 +2496,7 @@
     <row r="536">
       <c r="A536" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2504,7 +2504,7 @@
     <row r="538">
       <c r="A538" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2512,7 @@
     <row r="540">
       <c r="A540" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2585,7 +2585,7 @@
     <row r="559">
       <c r="A559" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2593,7 +2593,7 @@
     <row r="561">
       <c r="A561" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2601,7 @@
     <row r="563">
       <c r="A563" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2674,7 +2674,7 @@
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2682,7 +2682,7 @@
     <row r="584">
       <c r="A584" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2690,7 +2690,7 @@
     <row r="586">
       <c r="A586" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2763,7 +2763,7 @@
     <row r="605">
       <c r="A605" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2771,7 +2771,7 @@
     <row r="607">
       <c r="A607" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2779,7 +2779,7 @@
     <row r="609">
       <c r="A609" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2852,7 +2852,7 @@
     <row r="628">
       <c r="A628" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -2860,7 +2860,7 @@
     <row r="630">
       <c r="A630" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
     <row r="632">
       <c r="A632" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -2949,7 +2949,7 @@
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -2957,7 +2957,7 @@
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3038,7 +3038,7 @@
     <row r="676">
       <c r="A676" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3046,7 +3046,7 @@
     <row r="678">
       <c r="A678" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3119,7 +3119,7 @@
     <row r="697">
       <c r="A697" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3127,7 +3127,7 @@
     <row r="699">
       <c r="A699" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3135,7 +3135,7 @@
     <row r="701">
       <c r="A701" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
     <row r="720">
       <c r="A720" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3216,7 +3216,7 @@
     <row r="722">
       <c r="A722" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3224,7 @@
     <row r="724">
       <c r="A724" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3297,7 +3297,7 @@
     <row r="743">
       <c r="A743" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3305,7 @@
     <row r="745">
       <c r="A745" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3313,7 @@
     <row r="747">
       <c r="A747" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey and Finley./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey and Finley./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3386,7 +3386,7 @@
     <row r="766">
       <c r="A766" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3394,7 @@
     <row r="768">
       <c r="A768" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3402,7 +3402,7 @@
     <row r="770">
       <c r="A770" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3475,7 +3475,7 @@
     <row r="789">
       <c r="A789" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3483,7 +3483,7 @@
     <row r="791">
       <c r="A791" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3491,7 @@
     <row r="793">
       <c r="A793" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
     <row r="812">
       <c r="A812" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3572,7 +3572,7 @@
     <row r="814">
       <c r="A814" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3580,7 @@
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3653,7 +3653,7 @@
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3661,7 +3661,7 @@
     <row r="837">
       <c r="A837" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3669,7 +3669,7 @@
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3742,7 +3742,7 @@
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3750,7 @@
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3758,7 +3758,7 @@
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -3831,7 +3831,7 @@
     <row r="881">
       <c r="A881" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3839,7 @@
     <row r="883">
       <c r="A883" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -3847,7 +3847,7 @@
     <row r="885">
       <c r="A885" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -3920,7 +3920,7 @@
     <row r="904">
       <c r="A904" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -3928,7 +3928,7 @@
     <row r="906">
       <c r="A906" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -3936,7 +3936,7 @@
     <row r="908">
       <c r="A908" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4009,7 +4009,7 @@
     <row r="927">
       <c r="A927" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4017,7 @@
     <row r="929">
       <c r="A929" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4025,7 +4025,7 @@
     <row r="931">
       <c r="A931" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4098,7 +4098,7 @@
     <row r="950">
       <c r="A950" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4106,7 +4106,7 @@
     <row r="952">
       <c r="A952" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4114,7 +4114,7 @@
     <row r="954">
       <c r="A954" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Casey and Finley./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4187,7 +4187,7 @@
     <row r="973">
       <c r="A973" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4195,7 +4195,7 @@
     <row r="975">
       <c r="A975" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4203,7 +4203,7 @@
     <row r="977">
       <c r="A977" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4276,7 +4276,7 @@
     <row r="996">
       <c r="A996" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4284,7 +4284,7 @@
     <row r="998">
       <c r="A998" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4292,7 +4292,7 @@
     <row r="1000">
       <c r="A1000" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
     <row r="1019">
       <c r="A1019" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4373,7 +4373,7 @@
     <row r="1021">
       <c r="A1021" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4381,7 +4381,7 @@
     <row r="1023">
       <c r="A1023" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4454,7 +4454,7 @@
     <row r="1042">
       <c r="A1042" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4462,7 +4462,7 @@
     <row r="1044">
       <c r="A1044" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4470,7 +4470,7 @@
     <row r="1046">
       <c r="A1046" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4543,7 +4543,7 @@
     <row r="1065">
       <c r="A1065" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4551,7 +4551,7 @@
     <row r="1067">
       <c r="A1067" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4559,7 +4559,7 @@
     <row r="1069">
       <c r="A1069" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4632,7 +4632,7 @@
     <row r="1088">
       <c r="A1088" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4640,7 +4640,7 @@
     <row r="1090">
       <c r="A1090" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4648,7 +4648,7 @@
     <row r="1092">
       <c r="A1092" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4721,7 +4721,7 @@
     <row r="1111">
       <c r="A1111" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4729,7 +4729,7 @@
     <row r="1113">
       <c r="A1113" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4737,7 +4737,7 @@
     <row r="1115">
       <c r="A1115" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -4810,7 +4810,7 @@
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4818,7 +4818,7 @@
     <row r="1136">
       <c r="A1136" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
     <row r="1138">
       <c r="A1138" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4899,7 +4899,7 @@
     <row r="1157">
       <c r="A1157" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 06:45; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
     <row r="1159">
       <c r="A1159" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -4915,7 +4915,7 @@
     <row r="1161">
       <c r="A1161" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -4988,7 +4988,7 @@
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5004,7 +5004,7 @@
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5077,7 +5077,7 @@
     <row r="1203">
       <c r="A1203" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5085,7 +5085,7 @@
     <row r="1205">
       <c r="A1205" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5093,7 +5093,7 @@
     <row r="1207">
       <c r="A1207" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5166,7 +5166,7 @@
     <row r="1226">
       <c r="A1226" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5182,7 +5182,7 @@
     <row r="1230">
       <c r="A1230" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5255,7 +5255,7 @@
     <row r="1249">
       <c r="A1249" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5263,7 +5263,7 @@
     <row r="1251">
       <c r="A1251" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
     <row r="1253">
       <c r="A1253" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5344,7 +5344,7 @@
     <row r="1272">
       <c r="A1272" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5352,7 +5352,7 @@
     <row r="1274">
       <c r="A1274" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5360,7 +5360,7 @@
     <row r="1276">
       <c r="A1276" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 06:45; Team: Casey and Finley./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 06:45; Team: Casey and Finley./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5433,7 +5433,7 @@
     <row r="1295">
       <c r="A1295" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5441,7 +5441,7 @@
     <row r="1297">
       <c r="A1297" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Blake and Emery./; Description: Clearance./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Blake and Emery./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
     <row r="1299">
       <c r="A1299" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
     <row r="1318">
       <c r="A1318" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5530,7 +5530,7 @@
     <row r="1320">
       <c r="A1320" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5538,7 +5538,7 @@
     <row r="1322">
       <c r="A1322" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5611,7 +5611,7 @@
     <row r="1341">
       <c r="A1341" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5619,7 +5619,7 @@
     <row r="1343">
       <c r="A1343" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5627,7 +5627,7 @@
     <row r="1345">
       <c r="A1345" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5700,7 +5700,7 @@
     <row r="1364">
       <c r="A1364" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 85m² Textured Ceiling Removal./</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
     <row r="1366">
       <c r="A1366" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5716,7 +5716,7 @@
     <row r="1368">
       <c r="A1368" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5789,7 +5789,7 @@
     <row r="1387">
       <c r="A1387" t="inlineStr">
         <is>
-          <t>- Location: 59 Site-H Street, Southport, Testville.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 85 Hinau Road, Karaka Vale.; Start time at 07:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5797,7 +5797,7 @@
     <row r="1389">
       <c r="A1389" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 08:00; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5805,7 +5805,7 @@
     <row r="1391">
       <c r="A1391" t="inlineStr">
         <is>
-          <t>- Location: 24 Site-C Street, Westley, Testville.; Start time at 07:30; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 30 Harakeke Drive, Mahoe Glen.; Start time at 07:30; Team: Casey and Finley./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -5878,7 +5878,7 @@
     <row r="1410">
       <c r="A1410" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5886,7 +5886,7 @@
     <row r="1412">
       <c r="A1412" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5894,7 +5894,7 @@
     <row r="1414">
       <c r="A1414" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:30; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5967,7 +5967,7 @@
     <row r="1433">
       <c r="A1433" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 08:00; Team: Alex, Drew, Gray and Harper./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -5975,7 +5975,7 @@
     <row r="1435">
       <c r="A1435" t="inlineStr">
         <is>
-          <t>- Location: 38 Site-E Street, Northby, Testville.; Start time at 07:00; Team: Blake and Emery./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 52 Tawa Terrace, Totara Ridge.; Start time at 07:00; Team: Blake and Emery./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5983,7 @@
     <row r="1437">
       <c r="A1437" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 07:00; Team: Casey, Finley and Jordan./; Description: Class A-/ 40m² Vinyl Flooring Removal./</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
     <row r="1456">
       <c r="A1456" t="inlineStr">
         <is>
-          <t>- Location: 31 Site-D Street, Southport, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 41 Pohutu Place, Kakapo Flats.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -6064,7 +6064,7 @@
     <row r="1458">
       <c r="A1458" t="inlineStr">
         <is>
-          <t>- Location: 45 Site-F Street, Eastham, Testville.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
+          <t>- Location: 63 Matai Grove, Wetapunga Park.; Start time at 06:45; Team: Blake, Emery and Indy./; Description: Class B-/ Waste Collection./</t>
         </is>
       </c>
     </row>
@@ -6072,7 +6072,7 @@
     <row r="1460">
       <c r="A1460" t="inlineStr">
         <is>
-          <t>- Location: 52 Site-G Street, Westley, Testville.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
+          <t>- Location: 74 Nikau Way, Piwakawaka Heights.; Start time at 06:45; Team: Casey, Finley and Jordan./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
     <row r="1479">
       <c r="A1479" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Alex, Drew, Gray and Harper./; Description: Clearance./</t>
         </is>
       </c>
     </row>
@@ -6153,7 +6153,7 @@
     <row r="1481">
       <c r="A1481" t="inlineStr">
         <is>
-          <t>- Location: 17 Site-B Street, Eastham, Testville.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 19 Rimu Crescent, Rata Hollow.; Start time at 07:30; Team: Blake, Emery and Indy./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>
@@ -6161,7 +6161,7 @@
     <row r="1483">
       <c r="A1483" t="inlineStr">
         <is>
-          <t>- Location: 10 Site-A Street, Northby, Testville.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
+          <t>- Location: 8 Kowhai Lane, Tui Bay.; Start time at 08:00; Team: Casey, Finley and Jordan./; Description: Class B-/ 30m² Cladding Removal./</t>
         </is>
       </c>
     </row>

</xml_diff>